<commit_message>
P: RP : RheinWegDE : add kino sheet in Wiesbaden.xlsx
</commit_message>
<xml_diff>
--- a/P(Path)/RP(Rhine-Path)/RheinWegDE/RheinWeg-Beispiel-Firma-22-02-2026.xlsx
+++ b/P(Path)/RP(Rhine-Path)/RheinWegDE/RheinWeg-Beispiel-Firma-22-02-2026.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10917"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{449ECDC0-EDB9-6949-84CE-4A73E8842E6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{355BFADA-3B32-3647-93E5-21317BB8DA57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19020" yWindow="7760" windowWidth="36720" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="218">
   <si>
     <t>Firmenname: Suzhou Jinluorui Electronic Technology Co., Ltd. Einheitlicher Sozialkreditcode: 91320509MADJQQWQ7J</t>
   </si>
@@ -271,9 +271,6 @@
     <t>2</t>
   </si>
   <si>
-    <t>Liu Chenglong</t>
-  </si>
-  <si>
     <t>Aufsicht</t>
   </si>
   <si>
@@ -608,9 +605,6 @@
   </si>
   <si>
     <t>Art des Begünstigten</t>
-  </si>
-  <si>
-    <t>Jin Suyan -- 100% -- Suzhou Jinluorui Electronic Technology Co., Ltd.</t>
   </si>
   <si>
     <t>Rechtsvertreter; Geschäftsführer</t>
@@ -696,6 +690,15 @@
   <si>
     <t>*Haftungsausschluss: Diese Daten wurden von RheinWeg auf Anfrage anhand öffentlich zugänglicher Informationen recherchiert. Sie dienen ausschließlich Ihrer Information und stellen keine ausdrückliche oder stillschweigende Meinung oder Garantie seitens RheinWeg dar. Die Daten dienen lediglich Ihrer Entscheidungsfindung. RheinWeg übernimmt keine Haftung für Folgen, die sich aus der Verwendung dieser Daten ergeben. 
 Kontakt: 0160-1168307 Geschäftliche Anfragen: rheinwegde@gmail.com</t>
+  </si>
+  <si>
+    <t>Surname Nachname</t>
+  </si>
+  <si>
+    <t>Surname Nachname 2</t>
+  </si>
+  <si>
+    <t>Surname Nachname -- 100% -- Suzhou Jinluorui Electronic Technology Co., Ltd.</t>
   </si>
 </sst>
 </file>
@@ -1178,11 +1181,11 @@
   <sheetData>
     <row r="1" spans="1:21" ht="75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="11" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="D1" s="12"/>
       <c r="E1" s="12"/>
@@ -1350,39 +1353,39 @@
   <sheetData>
     <row r="1" spans="1:8" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="C1" s="6" t="s">
         <v>191</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="D1" s="6" t="s">
         <v>192</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="E1" s="6" t="s">
         <v>193</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="F1" s="6" t="s">
         <v>194</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="G1" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="H1" s="6" t="s">
         <v>196</v>
-      </c>
-      <c r="G1" s="6" t="s">
-        <v>197</v>
-      </c>
-      <c r="H1" s="6" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>197</v>
+      </c>
+      <c r="B2" t="s">
+        <v>198</v>
+      </c>
+      <c r="C2" t="s">
         <v>199</v>
-      </c>
-      <c r="B2" t="s">
-        <v>200</v>
-      </c>
-      <c r="C2" t="s">
-        <v>201</v>
       </c>
       <c r="D2" t="s">
         <v>50</v>
@@ -1391,13 +1394,13 @@
         <v>23</v>
       </c>
       <c r="F2" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="G2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="H2" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
     </row>
   </sheetData>
@@ -1420,30 +1423,30 @@
   <sheetData>
     <row r="1" spans="1:5" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="C1" s="6" t="s">
         <v>204</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="D1" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="E1" s="6" t="s">
         <v>206</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>207</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>207</v>
+      </c>
+      <c r="B2" t="s">
+        <v>208</v>
+      </c>
+      <c r="C2" t="s">
         <v>209</v>
-      </c>
-      <c r="B2" t="s">
-        <v>210</v>
-      </c>
-      <c r="C2" t="s">
-        <v>211</v>
       </c>
       <c r="D2" t="s">
         <v>32</v>
@@ -1472,30 +1475,30 @@
   <sheetData>
     <row r="1" spans="1:5" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="C1" s="6" t="s">
         <v>204</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="D1" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="E1" s="6" t="s">
         <v>206</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>207</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>210</v>
+      </c>
+      <c r="B2" t="s">
+        <v>211</v>
+      </c>
+      <c r="C2" t="s">
         <v>212</v>
-      </c>
-      <c r="B2" t="s">
-        <v>213</v>
-      </c>
-      <c r="C2" t="s">
-        <v>214</v>
       </c>
       <c r="D2" t="s">
         <v>32</v>
@@ -1532,7 +1535,7 @@
         <v>17</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>18</v>
+        <v>215</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="40" customHeight="1" x14ac:dyDescent="0.2">
@@ -1760,7 +1763,7 @@
     </row>
     <row r="3" spans="1:7" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>215</v>
       </c>
       <c r="B3" t="s">
         <v>64</v>
@@ -1792,7 +1795,8 @@
   <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="20" defaultRowHeight="26.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="15" customWidth="1"/>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="20.1640625" customWidth="1"/>
     <col min="3" max="3" width="30" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
     <col min="5" max="5" width="15" customWidth="1"/>
@@ -1824,7 +1828,7 @@
         <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>215</v>
       </c>
       <c r="C3" t="s">
         <v>68</v>
@@ -1838,10 +1842,10 @@
         <v>74</v>
       </c>
       <c r="B4" t="s">
+        <v>216</v>
+      </c>
+      <c r="C4" t="s">
         <v>75</v>
-      </c>
-      <c r="C4" t="s">
-        <v>76</v>
       </c>
       <c r="D4" t="s">
         <v>32</v>
@@ -1863,7 +1867,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
@@ -1890,63 +1894,63 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>77</v>
+      </c>
+      <c r="B4" t="s">
         <v>78</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>79</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>80</v>
-      </c>
-      <c r="D4" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
+        <v>81</v>
+      </c>
+      <c r="B5" t="s">
         <v>82</v>
-      </c>
-      <c r="B5" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>83</v>
+      </c>
+      <c r="B6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" t="s">
         <v>84</v>
       </c>
-      <c r="B6" t="s">
-        <v>32</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>85</v>
-      </c>
-      <c r="D6" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>86</v>
+      </c>
+      <c r="B7" t="s">
         <v>87</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>88</v>
       </c>
-      <c r="C7" t="s">
-        <v>89</v>
-      </c>
       <c r="D7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>89</v>
+      </c>
+      <c r="B8" t="s">
+        <v>85</v>
+      </c>
+      <c r="C8" t="s">
         <v>90</v>
-      </c>
-      <c r="B8" t="s">
-        <v>86</v>
-      </c>
-      <c r="C8" t="s">
-        <v>91</v>
       </c>
       <c r="D8" t="s">
         <v>32</v>
@@ -1954,30 +1958,30 @@
     </row>
     <row r="9" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
+        <v>92</v>
+      </c>
+      <c r="B10" t="s">
         <v>93</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>94</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>95</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>96</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
         <v>97</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>98</v>
-      </c>
-      <c r="G10" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
@@ -1985,13 +1989,13 @@
         <v>18</v>
       </c>
       <c r="B11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C11" t="s">
         <v>67</v>
       </c>
       <c r="D11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E11" t="s">
         <v>32</v>
@@ -2005,32 +2009,32 @@
     </row>
     <row r="12" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B13" t="s">
         <v>39</v>
       </c>
       <c r="C13" t="s">
+        <v>103</v>
+      </c>
+      <c r="D13" t="s">
         <v>104</v>
-      </c>
-      <c r="D13" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B14" t="s">
         <v>39</v>
       </c>
       <c r="C14" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D14" t="s">
         <v>39</v>
@@ -2038,7 +2042,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B15" t="s">
         <v>39</v>
@@ -2046,185 +2050,185 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
+        <v>108</v>
+      </c>
+      <c r="B16" t="s">
         <v>109</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
         <v>110</v>
-      </c>
-      <c r="C16" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
+        <v>111</v>
+      </c>
+      <c r="B17" t="s">
         <v>112</v>
       </c>
-      <c r="B17" t="s">
-        <v>113</v>
-      </c>
       <c r="C17" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B18" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C18" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B19" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C19" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
+        <v>115</v>
+      </c>
+      <c r="B20" t="s">
         <v>116</v>
       </c>
-      <c r="B20" t="s">
-        <v>117</v>
-      </c>
       <c r="C20" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B21" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C21" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B22" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C22" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B23" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C23" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B24" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C24" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
+        <v>120</v>
+      </c>
+      <c r="B25" t="s">
         <v>121</v>
       </c>
-      <c r="B25" t="s">
-        <v>122</v>
-      </c>
       <c r="C25" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B26" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C26" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B27" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C27" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B28" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C28" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B29" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C29" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="19" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
+        <v>126</v>
+      </c>
+      <c r="B31" t="s">
         <v>127</v>
-      </c>
-      <c r="B31" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="19" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
+        <v>129</v>
+      </c>
+      <c r="B33" t="s">
+        <v>32</v>
+      </c>
+      <c r="C33" t="s">
         <v>130</v>
-      </c>
-      <c r="B33" t="s">
-        <v>32</v>
-      </c>
-      <c r="C33" t="s">
-        <v>131</v>
       </c>
       <c r="D33" t="s">
         <v>32</v>
@@ -2232,13 +2236,13 @@
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
+        <v>131</v>
+      </c>
+      <c r="B34" t="s">
+        <v>32</v>
+      </c>
+      <c r="C34" t="s">
         <v>132</v>
-      </c>
-      <c r="B34" t="s">
-        <v>32</v>
-      </c>
-      <c r="C34" t="s">
-        <v>133</v>
       </c>
       <c r="D34" t="s">
         <v>32</v>
@@ -2246,13 +2250,13 @@
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
+        <v>133</v>
+      </c>
+      <c r="B35" t="s">
+        <v>32</v>
+      </c>
+      <c r="C35" t="s">
         <v>134</v>
-      </c>
-      <c r="B35" t="s">
-        <v>32</v>
-      </c>
-      <c r="C35" t="s">
-        <v>135</v>
       </c>
       <c r="D35" t="s">
         <v>32</v>
@@ -2260,13 +2264,13 @@
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
+        <v>135</v>
+      </c>
+      <c r="B36" t="s">
+        <v>32</v>
+      </c>
+      <c r="C36" t="s">
         <v>136</v>
-      </c>
-      <c r="B36" t="s">
-        <v>32</v>
-      </c>
-      <c r="C36" t="s">
-        <v>137</v>
       </c>
       <c r="D36" t="s">
         <v>32</v>
@@ -2274,38 +2278,38 @@
     </row>
     <row r="37" spans="1:8" ht="19" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
+        <v>138</v>
+      </c>
+      <c r="B38" t="s">
         <v>139</v>
       </c>
-      <c r="B38" t="s">
+      <c r="C38" t="s">
         <v>140</v>
       </c>
-      <c r="C38" t="s">
+      <c r="D38" t="s">
         <v>141</v>
       </c>
-      <c r="D38" t="s">
+      <c r="E38" t="s">
         <v>142</v>
       </c>
-      <c r="E38" t="s">
+      <c r="F38" t="s">
         <v>143</v>
       </c>
-      <c r="F38" t="s">
+      <c r="G38" t="s">
         <v>144</v>
       </c>
-      <c r="G38" t="s">
+      <c r="H38" t="s">
         <v>145</v>
-      </c>
-      <c r="H38" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="19" x14ac:dyDescent="0.25">
       <c r="A39" s="4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
@@ -2313,35 +2317,35 @@
         <v>70</v>
       </c>
       <c r="B40" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C40" t="s">
+        <v>147</v>
+      </c>
+      <c r="D40" t="s">
         <v>148</v>
       </c>
-      <c r="D40" t="s">
+      <c r="E40" t="s">
         <v>149</v>
-      </c>
-      <c r="E40" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="19" x14ac:dyDescent="0.25">
       <c r="A41" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
+        <v>151</v>
+      </c>
+      <c r="B42" t="s">
         <v>152</v>
       </c>
-      <c r="B42" t="s">
+      <c r="C42" t="s">
         <v>153</v>
       </c>
-      <c r="C42" t="s">
+      <c r="D42" t="s">
         <v>154</v>
-      </c>
-      <c r="D42" t="s">
-        <v>155</v>
       </c>
     </row>
   </sheetData>
@@ -2361,24 +2365,24 @@
   <sheetData>
     <row r="1" spans="1:4" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>157</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>158</v>
+      </c>
+      <c r="B2" t="s">
         <v>159</v>
-      </c>
-      <c r="B2" t="s">
-        <v>160</v>
       </c>
       <c r="C2" t="s">
         <v>32</v>
@@ -2389,10 +2393,10 @@
     </row>
     <row r="3" spans="1:4" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B3" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C3" t="s">
         <v>32</v>
@@ -2403,10 +2407,10 @@
     </row>
     <row r="4" spans="1:4" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C4" t="s">
         <v>32</v>
@@ -2437,19 +2441,19 @@
         <v>70</v>
       </c>
       <c r="B1" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="C1" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="D1" s="6" t="s">
         <v>164</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="E1" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="F1" s="6" t="s">
         <v>166</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -2457,19 +2461,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>18</v>
+        <v>215</v>
       </c>
       <c r="C2" s="13" t="s">
+        <v>167</v>
+      </c>
+      <c r="D2" s="13" t="s">
         <v>168</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="E2" s="13" t="s">
         <v>169</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="F2" t="s">
         <v>170</v>
-      </c>
-      <c r="F2" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -2479,7 +2483,7 @@
       <c r="D3" s="13"/>
       <c r="E3" s="13"/>
       <c r="F3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -2487,19 +2491,19 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>75</v>
+        <v>216</v>
       </c>
       <c r="C4" t="s">
+        <v>167</v>
+      </c>
+      <c r="D4" t="s">
         <v>168</v>
       </c>
-      <c r="D4" t="s">
-        <v>169</v>
-      </c>
       <c r="E4" t="s">
+        <v>172</v>
+      </c>
+      <c r="F4" t="s">
         <v>173</v>
-      </c>
-      <c r="F4" t="s">
-        <v>174</v>
       </c>
     </row>
   </sheetData>
@@ -2526,21 +2530,21 @@
   <sheetData>
     <row r="1" spans="1:4" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="C1" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="D1" s="6" t="s">
         <v>177</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="13" t="s">
-        <v>18</v>
+        <v>215</v>
       </c>
       <c r="B2" s="13" t="s">
         <v>64</v>
@@ -2549,7 +2553,7 @@
         <v>64</v>
       </c>
       <c r="D2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -2569,80 +2573,80 @@
   <sheetData>
     <row r="1" spans="1:5" s="2" customFormat="1" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="C2" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="D2" s="6" t="s">
         <v>182</v>
       </c>
-      <c r="C2" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>183</v>
-      </c>
       <c r="E2" s="6" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="13" t="s">
-        <v>18</v>
+        <v>215</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C3" s="13" t="s">
         <v>64</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="2" customFormat="1" ht="19" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="19" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="13" t="s">
-        <v>18</v>
+        <v>215</v>
       </c>
       <c r="B8" t="s">
-        <v>188</v>
+        <v>217</v>
       </c>
       <c r="C8" s="13" t="s">
         <v>64</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
   </sheetData>

</xml_diff>